<commit_message>
Ajout Bundle  Flux Alimentation (#49)
* correct fsh 3.0.0 errors

* add bundle flux alimentation profile

* add profile link in md and add Ressource Conformité in header

* add CI link on readme da78dd6379ec75ef23583b0bfb787a75993d07cb
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-observation-head-circumference.xlsx
+++ b/ig/main/StructureDefinition-mesures-observation-head-circumference.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-07-18T09:34:49+00:00</t>
+    <t>2023-07-18T09:37:51+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1245,12 +1245,6 @@
     <t>9. SHALL contain exactly one [1..1] value with @xsi:type="PQ" (CONF:7305).</t>
   </si>
   <si>
-    <t>&lt;valueQuantity xmlns="http://hl7.org/fhir"&gt;
-  &lt;system value="http://unitsofmeasure.org"/&gt;
-  &lt;code value="cm"/&gt;
-&lt;/valueQuantity&gt;</t>
-  </si>
-  <si>
     <t>ele-1
 obs-7vs-2</t>
   </si>
@@ -1368,6 +1362,9 @@
   </si>
   <si>
     <t>Need to know the system that defines the coded form of the unit.</t>
+  </si>
+  <si>
+    <t>http://unitsofmeasure.org</t>
   </si>
   <si>
     <t>Quantity.system</t>
@@ -8975,7 +8972,7 @@
         <v>36</v>
       </c>
       <c r="S56" t="s" s="2">
-        <v>392</v>
+        <v>36</v>
       </c>
       <c r="T56" t="s" s="2">
         <v>36</v>
@@ -9023,7 +9020,7 @@
         <v>46</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>59</v>
@@ -9032,27 +9029,27 @@
         <v>36</v>
       </c>
       <c r="AL56" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="AM56" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="AM56" t="s" s="2">
+      <c r="AN56" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="AN56" t="s" s="2">
+      <c r="AO56" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AP56" t="s" s="2">
         <v>396</v>
-      </c>
-      <c r="AO56" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AP56" t="s" s="2">
-        <v>397</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -9167,10 +9164,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9287,10 +9284,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9313,19 +9310,19 @@
         <v>47</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="L59" t="s" s="2">
         <v>401</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="M59" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="M59" t="s" s="2">
+      <c r="N59" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="N59" t="s" s="2">
+      <c r="O59" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="O59" t="s" s="2">
-        <v>405</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>36</v>
@@ -9374,7 +9371,7 @@
         <v>36</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>34</v>
@@ -9395,10 +9392,10 @@
         <v>36</v>
       </c>
       <c r="AM59" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="AN59" t="s" s="2">
         <v>407</v>
-      </c>
-      <c r="AN59" t="s" s="2">
-        <v>408</v>
       </c>
       <c r="AO59" t="s" s="2">
         <v>36</v>
@@ -9409,10 +9406,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9438,22 +9435,22 @@
         <v>126</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="N60" t="s" s="2">
         <v>261</v>
       </c>
       <c r="O60" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="P60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="Q60" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="P60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="Q60" t="s" s="2">
-        <v>413</v>
       </c>
       <c r="R60" t="s" s="2">
         <v>36</v>
@@ -9477,28 +9474,28 @@
         <v>200</v>
       </c>
       <c r="Y60" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="Z60" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="Z60" t="s" s="2">
+      <c r="AA60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AF60" t="s" s="2">
         <v>415</v>
-      </c>
-      <c r="AA60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AB60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AC60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AD60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AE60" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AF60" t="s" s="2">
-        <v>416</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>34</v>
@@ -9519,10 +9516,10 @@
         <v>36</v>
       </c>
       <c r="AM60" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="AN60" t="s" s="2">
         <v>417</v>
-      </c>
-      <c r="AN60" t="s" s="2">
-        <v>418</v>
       </c>
       <c r="AO60" t="s" s="2">
         <v>36</v>
@@ -9533,10 +9530,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9562,16 +9559,16 @@
         <v>62</v>
       </c>
       <c r="L61" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="M61" t="s" s="2">
         <v>420</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>421</v>
       </c>
       <c r="N61" t="s" s="2">
         <v>261</v>
       </c>
       <c r="O61" t="s" s="2">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>36</v>
@@ -9581,46 +9578,46 @@
         <v>36</v>
       </c>
       <c r="S61" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="Y61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="Z61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AA61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AB61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AC61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AD61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AE61" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AF61" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="T61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="U61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="V61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="W61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="X61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="Y61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="Z61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AA61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AB61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AC61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AD61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AE61" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AF61" t="s" s="2">
-        <v>424</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>34</v>
@@ -9641,10 +9638,10 @@
         <v>36</v>
       </c>
       <c r="AM61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="AN61" t="s" s="2">
         <v>425</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>426</v>
       </c>
       <c r="AO61" t="s" s="2">
         <v>36</v>
@@ -9655,10 +9652,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9666,7 +9663,7 @@
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s" s="2">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G62" t="s" s="2">
         <v>46</v>
@@ -9684,16 +9681,16 @@
         <v>90</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="M62" t="s" s="2">
         <v>428</v>
       </c>
-      <c r="M62" t="s" s="2">
+      <c r="N62" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="N62" t="s" s="2">
+      <c r="O62" t="s" s="2">
         <v>430</v>
-      </c>
-      <c r="O62" t="s" s="2">
-        <v>431</v>
       </c>
       <c r="P62" t="s" s="2">
         <v>36</v>
@@ -9703,7 +9700,7 @@
         <v>36</v>
       </c>
       <c r="S62" t="s" s="2">
-        <v>36</v>
+        <v>431</v>
       </c>
       <c r="T62" t="s" s="2">
         <v>36</v>
@@ -9763,7 +9760,7 @@
         <v>36</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AN62" t="s" s="2">
         <v>434</v>
@@ -9885,7 +9882,7 @@
         <v>36</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>441</v>
@@ -12907,16 +12904,16 @@
         <v>603</v>
       </c>
       <c r="AM88" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AN88" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="AN88" t="s" s="2">
+      <c r="AO88" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="AP88" t="s" s="2">
         <v>396</v>
-      </c>
-      <c r="AO88" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AP88" t="s" s="2">
-        <v>397</v>
       </c>
     </row>
     <row r="89" hidden="true">

</xml_diff>